<commit_message>
Correcciones en archivo de casos de prueba
</commit_message>
<xml_diff>
--- a/Pruebas_UniFootball_v2.xlsx
+++ b/Pruebas_UniFootball_v2.xlsx
@@ -4918,17 +4918,17 @@
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Compatibilidad de navegadores - Chrome, Firefox, Edge y Safari</t>
+          <t>Compatibilidad de navegadores - Chrome, Edge, Firefox y Opera</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>Build de la app accesible desde varios navegadores</t>
+          <t>Frontend (npm run dev) y backend corriendo en local; navegadores Chrome, Edge, Firefox y Opera instalados</t>
         </is>
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>1. Ejecutar el flujo core en Chrome (ultima y ultima-1) y Firefox</t>
+          <t>1. Ejecutar el flujo core (login, dashboard, equipos, torneos+detalle, navbar/logout) en Chrome y Edge (Chromium)</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
@@ -4936,7 +4936,11 @@
           <t>La app funciona y se ve correctamente</t>
         </is>
       </c>
-      <c r="H93" s="7" t="n"/>
+      <c r="H93" s="7" t="inlineStr">
+        <is>
+          <t>Analisis estatico: el front NO usa APIs especificas de navegador (sin navigator.* propietario, structuredClone, crypto.randomUUID), NI CSS con vendor prefixes / :has() / backdrop-filter / aspect-ratio; layout con Flexbox+Grid (soporte universal). Unica API moderna: Array.prototype.at() (Chrome/Edge/Firefox/Opera 2022+). Build de Vite a ES modules. =&gt; sin incompatibilidades de codigo. Confirmacion visual manual: guia Compatibilidad-8.2-Manual-UniFootball.md (matriz por navegador). Safari sustituido por Opera (equipo en Windows; se cubren motores Chromium y Gecko).</t>
+        </is>
+      </c>
       <c r="I93" s="7" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -4976,7 +4980,7 @@
       <c r="E94" s="8" t="n"/>
       <c r="F94" s="7" t="inlineStr">
         <is>
-          <t>2. Repetir en Edge (ultima) y Safari (macOS/iOS)</t>
+          <t>2. Repetir el mismo flujo en Firefox (Gecko) y Opera, revisando consola (F12) sin errores</t>
         </is>
       </c>
       <c r="G94" s="7" t="inlineStr">
@@ -5015,12 +5019,12 @@
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>Tests de Cypress/Playwright ejecutados en multiples viewports</t>
+          <t>Frontend corriendo en local; DevTools del navegador (Ctrl+Shift+M) para fijar viewports</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>1. Cargar la app en 1920x1080, 1440x900 y 1280x720 (desktop)</t>
+          <t>1. Cargar la app en 1920x1080, 1440x900 y 1280x720 (desktop) verificando sin scroll horizontal ni solapamientos</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
@@ -5028,7 +5032,11 @@
           <t>Layout correcto sin scroll horizontal ni solapamientos</t>
         </is>
       </c>
-      <c r="H95" s="7" t="n"/>
+      <c r="H95" s="7" t="inlineStr">
+        <is>
+          <t>Prueba manual con DevTools (toggle device toolbar). Layout responsive basado en Flexbox/Grid sin medidas fijas que rompan en movil. Matriz de 6 viewports (3 desktop + 1 tablet + 2 movil) en la guia Compatibilidad-8.2-Manual-UniFootball.md para registrar layout / sin scroll horizontal / usabilidad por viewport.</t>
+        </is>
+      </c>
       <c r="I95" s="7" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -5068,7 +5076,7 @@
       <c r="E96" s="8" t="n"/>
       <c r="F96" s="7" t="inlineStr">
         <is>
-          <t>2. Cargar en 768x1024 (iPad) y 390x844 / 360x800 (movil)</t>
+          <t>2. Repetir en 768x1024 (tablet) y 390x844 / 360x800 (movil), verificando UI responsive y usable</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
@@ -6057,8 +6065,8 @@
   <autoFilter ref="A1:N163"/>
   <mergeCells count="506">
     <mergeCell ref="I32:I33"/>
+    <mergeCell ref="K32:K33"/>
     <mergeCell ref="J60:J61"/>
-    <mergeCell ref="K32:K33"/>
     <mergeCell ref="D21:D22"/>
     <mergeCell ref="M54:M55"/>
     <mergeCell ref="B23:B24"/>
@@ -6087,11 +6095,11 @@
     <mergeCell ref="N41:N42"/>
     <mergeCell ref="B77:B78"/>
     <mergeCell ref="A45:A46"/>
+    <mergeCell ref="D17:D18"/>
     <mergeCell ref="D77:D78"/>
     <mergeCell ref="M47:M49"/>
     <mergeCell ref="D11:D12"/>
     <mergeCell ref="I7:I8"/>
-    <mergeCell ref="D17:D18"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="C45:C46"/>
     <mergeCell ref="L43:L44"/>
@@ -6100,8 +6108,8 @@
     <mergeCell ref="D75:D76"/>
     <mergeCell ref="I71:I72"/>
     <mergeCell ref="K71:K72"/>
+    <mergeCell ref="J99:J100"/>
     <mergeCell ref="I65:I67"/>
-    <mergeCell ref="J99:J100"/>
     <mergeCell ref="M29:M31"/>
     <mergeCell ref="K65:K67"/>
     <mergeCell ref="A89:A90"/>
@@ -6122,9 +6130,9 @@
     <mergeCell ref="M43:M44"/>
     <mergeCell ref="N54:N55"/>
     <mergeCell ref="L29:L31"/>
-    <mergeCell ref="C2:C4"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="N56:N57"/>
+    <mergeCell ref="C2:C4"/>
     <mergeCell ref="M11:M12"/>
     <mergeCell ref="A41:A42"/>
     <mergeCell ref="J87:J88"/>
@@ -6144,9 +6152,9 @@
     <mergeCell ref="N9:N10"/>
     <mergeCell ref="D83:D84"/>
     <mergeCell ref="K73:K74"/>
+    <mergeCell ref="D93:D94"/>
+    <mergeCell ref="I23:I24"/>
     <mergeCell ref="B2:B4"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="D93:D94"/>
     <mergeCell ref="A97:A98"/>
     <mergeCell ref="L77:L78"/>
     <mergeCell ref="L11:L12"/>
@@ -6161,12 +6169,12 @@
     <mergeCell ref="N29:N31"/>
     <mergeCell ref="E34:E35"/>
     <mergeCell ref="D38:D40"/>
+    <mergeCell ref="D91:D92"/>
     <mergeCell ref="I21:I22"/>
-    <mergeCell ref="D91:D92"/>
     <mergeCell ref="A95:A96"/>
     <mergeCell ref="I5:I6"/>
+    <mergeCell ref="A5:A6"/>
     <mergeCell ref="A32:A33"/>
-    <mergeCell ref="A5:A6"/>
     <mergeCell ref="E68:E70"/>
     <mergeCell ref="K23:K24"/>
     <mergeCell ref="E36:E37"/>
@@ -6174,12 +6182,12 @@
     <mergeCell ref="M2:M4"/>
     <mergeCell ref="K87:K88"/>
     <mergeCell ref="M87:M88"/>
-    <mergeCell ref="L17:L18"/>
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="M56:M57"/>
+    <mergeCell ref="L17:L18"/>
     <mergeCell ref="B41:B42"/>
+    <mergeCell ref="J19:J20"/>
     <mergeCell ref="L19:L20"/>
-    <mergeCell ref="J19:J20"/>
     <mergeCell ref="L75:L76"/>
     <mergeCell ref="N75:N76"/>
     <mergeCell ref="B43:B44"/>
@@ -6188,8 +6196,8 @@
     <mergeCell ref="D99:D100"/>
     <mergeCell ref="N25:N26"/>
     <mergeCell ref="N85:N86"/>
+    <mergeCell ref="B68:B70"/>
     <mergeCell ref="K89:K90"/>
-    <mergeCell ref="B68:B70"/>
     <mergeCell ref="D68:D70"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="L83:L84"/>
@@ -6211,7 +6219,6 @@
     <mergeCell ref="B54:B55"/>
     <mergeCell ref="I50:I51"/>
     <mergeCell ref="D54:D55"/>
-    <mergeCell ref="D71:D72"/>
     <mergeCell ref="B56:B57"/>
     <mergeCell ref="L38:L40"/>
     <mergeCell ref="D34:D35"/>
@@ -6227,17 +6234,17 @@
     <mergeCell ref="J91:J92"/>
     <mergeCell ref="L2:L4"/>
     <mergeCell ref="N13:N14"/>
-    <mergeCell ref="C17:C18"/>
     <mergeCell ref="K17:K18"/>
     <mergeCell ref="A17:A18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="L34:L35"/>
     <mergeCell ref="L47:L49"/>
-    <mergeCell ref="L34:L35"/>
     <mergeCell ref="N47:N49"/>
     <mergeCell ref="L99:L100"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="N15:N16"/>
     <mergeCell ref="K19:K20"/>
     <mergeCell ref="A19:A20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="N15:N16"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="A43:A44"/>
     <mergeCell ref="N79:N80"/>
@@ -6261,10 +6268,10 @@
     <mergeCell ref="M75:M76"/>
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="A13:A14"/>
+    <mergeCell ref="L41:L42"/>
+    <mergeCell ref="C7:C8"/>
     <mergeCell ref="E7:E8"/>
-    <mergeCell ref="C7:C8"/>
     <mergeCell ref="I47:I49"/>
-    <mergeCell ref="L41:L42"/>
     <mergeCell ref="J43:J44"/>
     <mergeCell ref="E71:E72"/>
     <mergeCell ref="J5:J6"/>
@@ -6323,9 +6330,11 @@
     <mergeCell ref="B47:B49"/>
     <mergeCell ref="E89:E90"/>
     <mergeCell ref="I43:I44"/>
+    <mergeCell ref="B15:B16"/>
     <mergeCell ref="K43:K44"/>
-    <mergeCell ref="B15:B16"/>
     <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D71:D72"/>
+    <mergeCell ref="C43:C44"/>
     <mergeCell ref="D65:D67"/>
     <mergeCell ref="J29:J31"/>
     <mergeCell ref="N62:N64"/>
@@ -6342,12 +6351,13 @@
     <mergeCell ref="I87:I88"/>
     <mergeCell ref="L58:L59"/>
     <mergeCell ref="L65:L67"/>
-    <mergeCell ref="K56:K57"/>
+    <mergeCell ref="N58:N59"/>
     <mergeCell ref="I56:I57"/>
     <mergeCell ref="N52:N53"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="K56:K57"/>
+    <mergeCell ref="M13:M14"/>
     <mergeCell ref="C56:C57"/>
-    <mergeCell ref="A56:A57"/>
-    <mergeCell ref="M13:M14"/>
     <mergeCell ref="M38:M40"/>
     <mergeCell ref="C62:C64"/>
     <mergeCell ref="C95:C96"/>
@@ -6364,16 +6374,16 @@
     <mergeCell ref="B79:B80"/>
     <mergeCell ref="D79:D80"/>
     <mergeCell ref="I9:I10"/>
+    <mergeCell ref="A9:A10"/>
     <mergeCell ref="C34:C35"/>
-    <mergeCell ref="A9:A10"/>
     <mergeCell ref="M52:M53"/>
     <mergeCell ref="D23:D24"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="L7:L8"/>
     <mergeCell ref="D81:D82"/>
     <mergeCell ref="I77:I78"/>
     <mergeCell ref="N7:N8"/>
     <mergeCell ref="I11:I12"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="B81:B82"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="L71:L72"/>
     <mergeCell ref="I75:I76"/>
@@ -6387,34 +6397,33 @@
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="L25:L26"/>
     <mergeCell ref="M45:M46"/>
-    <mergeCell ref="E32:E33"/>
     <mergeCell ref="M32:M33"/>
     <mergeCell ref="L60:L61"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="N60:N61"/>
     <mergeCell ref="B36:B37"/>
-    <mergeCell ref="N60:N61"/>
     <mergeCell ref="C91:C92"/>
     <mergeCell ref="A93:A94"/>
     <mergeCell ref="M58:M59"/>
-    <mergeCell ref="L13:L14"/>
     <mergeCell ref="J13:J14"/>
     <mergeCell ref="E17:E18"/>
+    <mergeCell ref="L13:L14"/>
     <mergeCell ref="J47:J49"/>
     <mergeCell ref="K60:K61"/>
     <mergeCell ref="M60:M61"/>
     <mergeCell ref="E19:E20"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="L15:L16"/>
-    <mergeCell ref="D5:D6"/>
     <mergeCell ref="N71:N72"/>
     <mergeCell ref="A75:A76"/>
     <mergeCell ref="C75:C76"/>
     <mergeCell ref="D95:D96"/>
     <mergeCell ref="I25:I26"/>
     <mergeCell ref="J79:J80"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="L79:L80"/>
     <mergeCell ref="C25:C26"/>
-    <mergeCell ref="A25:A26"/>
     <mergeCell ref="I83:I84"/>
-    <mergeCell ref="L79:L80"/>
     <mergeCell ref="L73:L74"/>
     <mergeCell ref="N73:N74"/>
     <mergeCell ref="L23:L24"/>
@@ -6424,8 +6433,8 @@
     <mergeCell ref="C52:C53"/>
     <mergeCell ref="N87:N88"/>
     <mergeCell ref="I13:I14"/>
+    <mergeCell ref="K13:K14"/>
     <mergeCell ref="E45:E46"/>
-    <mergeCell ref="K13:K14"/>
     <mergeCell ref="A81:A82"/>
     <mergeCell ref="J41:J42"/>
     <mergeCell ref="C81:C82"/>
@@ -6449,11 +6458,10 @@
     <mergeCell ref="D45:D46"/>
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="A68:A70"/>
-    <mergeCell ref="D32:D33"/>
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="A71:A72"/>
+    <mergeCell ref="D32:D33"/>
     <mergeCell ref="C71:C72"/>
-    <mergeCell ref="C43:C44"/>
     <mergeCell ref="J36:J37"/>
     <mergeCell ref="B62:B64"/>
     <mergeCell ref="M17:M18"/>
@@ -6465,12 +6473,12 @@
     <mergeCell ref="I99:I100"/>
     <mergeCell ref="N95:N96"/>
     <mergeCell ref="N89:N90"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="M50:M51"/>
     <mergeCell ref="I68:I70"/>
     <mergeCell ref="K15:K16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="M50:M51"/>
+    <mergeCell ref="B27:B28"/>
     <mergeCell ref="D27:D28"/>
-    <mergeCell ref="B27:B28"/>
     <mergeCell ref="K79:K80"/>
     <mergeCell ref="M79:M80"/>
     <mergeCell ref="J34:J35"/>
@@ -6492,9 +6500,9 @@
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="B38:B40"/>
     <mergeCell ref="K5:K6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="C5:C6"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="B71:B72"/>
     <mergeCell ref="B65:B67"/>
     <mergeCell ref="J62:J64"/>
@@ -6502,7 +6510,6 @@
     <mergeCell ref="I36:I37"/>
     <mergeCell ref="L97:L98"/>
     <mergeCell ref="A36:A37"/>
-    <mergeCell ref="N58:N59"/>
     <mergeCell ref="N97:N98"/>
     <mergeCell ref="B73:B74"/>
     <mergeCell ref="A62:A64"/>
@@ -6517,26 +6524,26 @@
     <mergeCell ref="J50:J51"/>
     <mergeCell ref="C29:C31"/>
     <mergeCell ref="N83:N84"/>
+    <mergeCell ref="L50:L51"/>
     <mergeCell ref="A65:A67"/>
-    <mergeCell ref="L50:L51"/>
     <mergeCell ref="B99:B100"/>
     <mergeCell ref="E29:E31"/>
     <mergeCell ref="K97:K98"/>
+    <mergeCell ref="J58:J59"/>
+    <mergeCell ref="M97:M98"/>
     <mergeCell ref="J52:J53"/>
     <mergeCell ref="E56:E57"/>
-    <mergeCell ref="J58:J59"/>
     <mergeCell ref="L52:L53"/>
-    <mergeCell ref="M97:M98"/>
     <mergeCell ref="A83:A84"/>
     <mergeCell ref="A58:A59"/>
+    <mergeCell ref="J81:J82"/>
     <mergeCell ref="B21:B22"/>
-    <mergeCell ref="J81:J82"/>
     <mergeCell ref="N45:N46"/>
     <mergeCell ref="N32:N33"/>
     <mergeCell ref="K36:K37"/>
     <mergeCell ref="K21:K22"/>
+    <mergeCell ref="A60:A61"/>
     <mergeCell ref="C89:C90"/>
-    <mergeCell ref="A60:A61"/>
     <mergeCell ref="K50:K51"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="E9:E10"/>
@@ -6555,8 +6562,9 @@
     <mergeCell ref="B89:B90"/>
     <mergeCell ref="D89:D90"/>
     <mergeCell ref="B5:B6"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="D5:D6"/>
     <mergeCell ref="N27:N28"/>
-    <mergeCell ref="L27:L28"/>
     <mergeCell ref="I62:I64"/>
     <mergeCell ref="C65:C67"/>
     <mergeCell ref="N2:N4"/>
@@ -7195,7 +7203,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -7236,7 +7243,6 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -7285,7 +7291,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -7298,7 +7303,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -7406,7 +7410,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Actualizar casos de prueba y registro de defectos (8.2, bug report)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pruebas_UniFootball_v2.xlsx
+++ b/Pruebas_UniFootball_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\OneDrive\Calidad de Software\unifootball\unifootball\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F805B8BD-2998-4891-8A60-BD5D130E53E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650761A9-9929-4923-91DF-DAF974A8C733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Casos de Prueba" sheetId="1" r:id="rId1"/>
     <sheet name="Registro de Defectos" sheetId="2" r:id="rId2"/>
     <sheet name="Resumen" sheetId="3" r:id="rId3"/>
-    <sheet name="Trazabilidad Examen" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Prueba'!$A$1:$N$163</definedName>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="588">
   <si>
     <t>Capa</t>
   </si>
@@ -1813,132 +1812,6 @@
   </si>
   <si>
     <t>Defectos identificados</t>
-  </si>
-  <si>
-    <t>Seccion del Examen (Checklist)</t>
-  </si>
-  <si>
-    <t>Requisito</t>
-  </si>
-  <si>
-    <t>Casos que lo cubren</t>
-  </si>
-  <si>
-    <t># Casos</t>
-  </si>
-  <si>
-    <t>1.2 Casos de Prueba</t>
-  </si>
-  <si>
-    <t>11 campos obligatorios por caso (ID, titulo, precondiciones, datos reales, pasos numerados, resultado esperado/real, status, severidad, prioridad, automatizado, requisito)</t>
-  </si>
-  <si>
-    <t>Estructura de columnas de la hoja 'Casos de Prueba'</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>3 Pruebas Unitarias</t>
-  </si>
-  <si>
-    <t>Logica de negocio, servicios y componentes UI en aislamiento (mocks)</t>
-  </si>
-  <si>
-    <t>TC-UNIT-001 a TC-UNIT-017</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>4.1 Integracion - API REST</t>
-  </si>
-  <si>
-    <t>Happy path, validaciones 400, auth 401, 404, 409, idempotencia, filtros, schema</t>
-  </si>
-  <si>
-    <t>TC-API-001..008, 010, 011</t>
-  </si>
-  <si>
-    <t>4.2 Integracion - BD Relacional</t>
-  </si>
-  <si>
-    <t>Constraints UNIQUE/NOT NULL/FK, CRUD de repos, transacciones, aislamiento, seed</t>
-  </si>
-  <si>
-    <t>TC-DBSQL-001, 002, 004, 006</t>
-  </si>
-  <si>
-    <t>4.3 Integracion - BD NoSQL</t>
-  </si>
-  <si>
-    <t>Validacion de schema, colecciones limpias, orden, documentos, indices</t>
-  </si>
-  <si>
-    <t>TC-DBNOSQL-001, 003, 004, 005</t>
-  </si>
-  <si>
-    <t>5 Pruebas End-to-End</t>
-  </si>
-  <si>
-    <t>Registro, login/logout, flujo core, roles, flujos de error, sesion</t>
-  </si>
-  <si>
-    <t>TC-E2E-001 a TC-E2E-006</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>6 Pruebas de Rendimiento</t>
-  </si>
-  <si>
-    <t>Load, Stress, Spike y Soak con k6</t>
-  </si>
-  <si>
-    <t>TC-PERF-001 a TC-PERF-004</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>7 Pruebas de Seguridad (OWASP Top 10)</t>
-  </si>
-  <si>
-    <t>A01 Access Control, A02 Crypto, A03 Injection/XSS, A05 Misconfig, A06 Componentes, A07 Auth</t>
-  </si>
-  <si>
-    <t>TC-SEC-003, 004, 006</t>
-  </si>
-  <si>
-    <t>8 Accesibilidad y Compatibilidad</t>
-  </si>
-  <si>
-    <t>WCAG 2.1 (teclado, alt, labels, aria) y cross-browser/responsive</t>
-  </si>
-  <si>
-    <t>TC-A11Y-001/002 y TC-COMPAT-001/002</t>
-  </si>
-  <si>
-    <t>11 Observabilidad / Monitoreo</t>
-  </si>
-  <si>
-    <t>Logs estructurados sin PII y metricas RED por endpoint</t>
-  </si>
-  <si>
-    <t>TC-OBS-001 a TC-OBS-002</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>1.3 Registro de Defectos</t>
-  </si>
-  <si>
-    <t>ID, titulo, descripcion actual/esperado, pasos, evidencia, severidad, prioridad, entorno, version, asignado, estado ciclo</t>
-  </si>
-  <si>
-    <t>Defectos en hoja Registro de Defectos (DEF-001 y DEF-007 descartados: no reproducibles)</t>
   </si>
   <si>
     <t>PASS</t>
@@ -2198,39 +2071,39 @@
     <xf numFmtId="0" fontId="4" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2598,19 +2471,19 @@
       </c>
     </row>
     <row r="2" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="18" t="s">
         <v>18</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -2620,31 +2493,31 @@
         <v>20</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" s="16" t="s">
+      <c r="I2" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="16" t="s">
+      <c r="J2" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="L2" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="16" t="s">
+      <c r="M2" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="N2" s="16" t="s">
+      <c r="N2" s="18" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="20"/>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
       <c r="F3" s="2" t="s">
         <v>27</v>
       </c>
@@ -2652,12 +2525,12 @@
         <v>28</v>
       </c>
       <c r="H3" s="2"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
     </row>
     <row r="4" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="17"/>
@@ -2680,19 +2553,19 @@
       <c r="N4" s="17"/>
     </row>
     <row r="5" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="18" t="s">
         <v>33</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -2702,22 +2575,22 @@
         <v>35</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="16" t="s">
+      <c r="K5" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L5" s="16" t="s">
+      <c r="L5" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M5" s="16" t="s">
+      <c r="M5" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="N5" s="16" t="s">
+      <c r="N5" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2742,19 +2615,19 @@
       <c r="N6" s="17"/>
     </row>
     <row r="7" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="18" t="s">
         <v>41</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -2764,22 +2637,22 @@
         <v>43</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="I7" s="16" t="s">
+      <c r="I7" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J7" s="16" t="s">
+      <c r="J7" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K7" s="16" t="s">
+      <c r="K7" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L7" s="16" t="s">
+      <c r="L7" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M7" s="16" t="s">
+      <c r="M7" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="N7" s="16" t="s">
+      <c r="N7" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2804,19 +2677,19 @@
       <c r="N8" s="17"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="18" t="s">
         <v>49</v>
       </c>
       <c r="F9" s="2" t="s">
@@ -2826,22 +2699,22 @@
         <v>51</v>
       </c>
       <c r="H9" s="2"/>
-      <c r="I9" s="16" t="s">
+      <c r="I9" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="J9" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K9" s="16" t="s">
+      <c r="K9" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L9" s="16" t="s">
+      <c r="L9" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="16" t="s">
+      <c r="M9" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="N9" s="16" t="s">
+      <c r="N9" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2866,19 +2739,19 @@
       <c r="N10" s="17"/>
     </row>
     <row r="11" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="18" t="s">
         <v>57</v>
       </c>
       <c r="F11" s="2" t="s">
@@ -2888,22 +2761,22 @@
         <v>59</v>
       </c>
       <c r="H11" s="2"/>
-      <c r="I11" s="16" t="s">
+      <c r="I11" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J11" s="16" t="s">
+      <c r="J11" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K11" s="16" t="s">
+      <c r="K11" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L11" s="16" t="s">
+      <c r="L11" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M11" s="16" t="s">
+      <c r="M11" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="N11" s="16" t="s">
+      <c r="N11" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2928,19 +2801,19 @@
       <c r="N12" s="17"/>
     </row>
     <row r="13" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="18" t="s">
         <v>64</v>
       </c>
       <c r="F13" s="2" t="s">
@@ -2950,22 +2823,22 @@
         <v>66</v>
       </c>
       <c r="H13" s="2"/>
-      <c r="I13" s="16" t="s">
+      <c r="I13" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K13" s="16" t="s">
+      <c r="K13" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L13" s="16" t="s">
+      <c r="L13" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M13" s="16" t="s">
+      <c r="M13" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="N13" s="16" t="s">
+      <c r="N13" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2990,19 +2863,19 @@
       <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="18" t="s">
         <v>72</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -3012,22 +2885,22 @@
         <v>74</v>
       </c>
       <c r="H15" s="2"/>
-      <c r="I15" s="16" t="s">
+      <c r="I15" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J15" s="16" t="s">
+      <c r="J15" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K15" s="16" t="s">
+      <c r="K15" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L15" s="16" t="s">
+      <c r="L15" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M15" s="16" t="s">
+      <c r="M15" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="N15" s="16" t="s">
+      <c r="N15" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3052,19 +2925,19 @@
       <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="18" t="s">
         <v>81</v>
       </c>
       <c r="F17" s="2" t="s">
@@ -3074,22 +2947,22 @@
         <v>83</v>
       </c>
       <c r="H17" s="2"/>
-      <c r="I17" s="16" t="s">
+      <c r="I17" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J17" s="16" t="s">
+      <c r="J17" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K17" s="16" t="s">
+      <c r="K17" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L17" s="16" t="s">
+      <c r="L17" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M17" s="16" t="s">
+      <c r="M17" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="N17" s="16" t="s">
+      <c r="N17" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3114,19 +2987,19 @@
       <c r="N18" s="17"/>
     </row>
     <row r="19" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="E19" s="18" t="s">
         <v>88</v>
       </c>
       <c r="F19" s="2" t="s">
@@ -3136,22 +3009,22 @@
         <v>90</v>
       </c>
       <c r="H19" s="2"/>
-      <c r="I19" s="16" t="s">
+      <c r="I19" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J19" s="16" t="s">
+      <c r="J19" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K19" s="16" t="s">
+      <c r="K19" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L19" s="16" t="s">
+      <c r="L19" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M19" s="16" t="s">
+      <c r="M19" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="N19" s="16" t="s">
+      <c r="N19" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3176,19 +3049,19 @@
       <c r="N20" s="17"/>
     </row>
     <row r="21" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="26" t="s">
+      <c r="A21" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="E21" s="16" t="s">
+      <c r="E21" s="18" t="s">
         <v>98</v>
       </c>
       <c r="F21" s="2" t="s">
@@ -3200,22 +3073,22 @@
       <c r="H21" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="I21" s="16" t="s">
+      <c r="I21" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J21" s="16" t="s">
+      <c r="J21" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K21" s="16" t="s">
+      <c r="K21" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="L21" s="16" t="s">
+      <c r="L21" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M21" s="16" t="s">
+      <c r="M21" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="N21" s="16" t="s">
+      <c r="N21" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3240,19 +3113,19 @@
       <c r="N22" s="17"/>
     </row>
     <row r="23" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="26" t="s">
+      <c r="A23" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="D23" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="E23" s="16" t="s">
+      <c r="E23" s="18" t="s">
         <v>107</v>
       </c>
       <c r="F23" s="2" t="s">
@@ -3264,22 +3137,22 @@
       <c r="H23" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="I23" s="16" t="s">
+      <c r="I23" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="16" t="s">
+      <c r="J23" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="16" t="s">
+      <c r="K23" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L23" s="16" t="s">
+      <c r="L23" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M23" s="16" t="s">
+      <c r="M23" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="N23" s="16" t="s">
+      <c r="N23" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3304,19 +3177,19 @@
       <c r="N24" s="17"/>
     </row>
     <row r="25" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="26" t="s">
+      <c r="A25" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="D25" s="16" t="s">
+      <c r="D25" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="E25" s="16" t="s">
+      <c r="E25" s="18" t="s">
         <v>116</v>
       </c>
       <c r="F25" s="2" t="s">
@@ -3328,22 +3201,22 @@
       <c r="H25" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I25" s="16" t="s">
+      <c r="I25" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J25" s="16" t="s">
+      <c r="J25" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K25" s="16" t="s">
+      <c r="K25" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L25" s="16" t="s">
+      <c r="L25" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M25" s="16" t="s">
+      <c r="M25" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="N25" s="16" t="s">
+      <c r="N25" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3368,19 +3241,19 @@
       <c r="N26" s="17"/>
     </row>
     <row r="27" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="26" t="s">
+      <c r="A27" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="D27" s="16" t="s">
+      <c r="D27" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="E27" s="16" t="s">
+      <c r="E27" s="18" t="s">
         <v>124</v>
       </c>
       <c r="F27" s="2" t="s">
@@ -3392,22 +3265,22 @@
       <c r="H27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="I27" s="16" t="s">
+      <c r="I27" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J27" s="16" t="s">
+      <c r="J27" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K27" s="16" t="s">
+      <c r="K27" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L27" s="16" t="s">
+      <c r="L27" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M27" s="16" t="s">
+      <c r="M27" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="N27" s="16" t="s">
+      <c r="N27" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3432,19 +3305,19 @@
       <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14" ht="116" x14ac:dyDescent="0.35">
-      <c r="A29" s="26" t="s">
+      <c r="A29" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="D29" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E29" s="18" t="s">
         <v>132</v>
       </c>
       <c r="F29" s="2" t="s">
@@ -3456,31 +3329,31 @@
       <c r="H29" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="I29" s="16" t="s">
+      <c r="I29" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J29" s="16" t="s">
+      <c r="J29" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K29" s="16" t="s">
+      <c r="K29" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L29" s="16" t="s">
+      <c r="L29" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M29" s="16" t="s">
+      <c r="M29" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="N29" s="16" t="s">
+      <c r="N29" s="18" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
+      <c r="A30" s="19"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
       <c r="F30" s="2" t="s">
         <v>136</v>
       </c>
@@ -3488,12 +3361,12 @@
         <v>137</v>
       </c>
       <c r="H30" s="2"/>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
-      <c r="L30" s="20"/>
-      <c r="M30" s="20"/>
-      <c r="N30" s="20"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="19"/>
+      <c r="K30" s="19"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="19"/>
+      <c r="N30" s="19"/>
     </row>
     <row r="31" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="17"/>
@@ -3516,19 +3389,19 @@
       <c r="N31" s="17"/>
     </row>
     <row r="32" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="26" t="s">
+      <c r="A32" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="D32" s="16" t="s">
+      <c r="D32" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="E32" s="16" t="s">
+      <c r="E32" s="18" t="s">
         <v>142</v>
       </c>
       <c r="F32" s="2" t="s">
@@ -3540,22 +3413,22 @@
       <c r="H32" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="I32" s="16" t="s">
+      <c r="I32" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J32" s="16" t="s">
+      <c r="J32" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K32" s="16" t="s">
+      <c r="K32" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L32" s="16" t="s">
+      <c r="L32" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M32" s="16" t="s">
+      <c r="M32" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="N32" s="16" t="s">
+      <c r="N32" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3580,19 +3453,19 @@
       <c r="N33" s="17"/>
     </row>
     <row r="34" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="26" t="s">
+      <c r="A34" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C34" s="16" t="s">
+      <c r="C34" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="D34" s="16" t="s">
+      <c r="D34" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="E34" s="16" t="s">
+      <c r="E34" s="18" t="s">
         <v>150</v>
       </c>
       <c r="F34" s="2" t="s">
@@ -3604,22 +3477,22 @@
       <c r="H34" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="I34" s="16" t="s">
+      <c r="I34" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J34" s="16" t="s">
+      <c r="J34" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K34" s="16" t="s">
+      <c r="K34" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L34" s="16" t="s">
+      <c r="L34" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M34" s="16" t="s">
+      <c r="M34" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="N34" s="16" t="s">
+      <c r="N34" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3644,19 +3517,19 @@
       <c r="N35" s="17"/>
     </row>
     <row r="36" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="26" t="s">
+      <c r="A36" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="D36" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="E36" s="16" t="s">
+      <c r="E36" s="18" t="s">
         <v>160</v>
       </c>
       <c r="F36" s="2" t="s">
@@ -3668,22 +3541,22 @@
       <c r="H36" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="I36" s="16" t="s">
+      <c r="I36" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J36" s="16" t="s">
+      <c r="J36" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K36" s="16" t="s">
+      <c r="K36" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L36" s="16" t="s">
+      <c r="L36" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M36" s="16" t="s">
+      <c r="M36" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="N36" s="16" t="s">
+      <c r="N36" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3708,19 +3581,19 @@
       <c r="N37" s="17"/>
     </row>
     <row r="38" spans="1:14" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="26" t="s">
+      <c r="A38" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="B38" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="D38" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="E38" s="16" t="s">
+      <c r="E38" s="18" t="s">
         <v>169</v>
       </c>
       <c r="F38" s="2" t="s">
@@ -3732,31 +3605,31 @@
       <c r="H38" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="I38" s="16" t="s">
+      <c r="I38" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J38" s="16" t="s">
+      <c r="J38" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K38" s="16" t="s">
+      <c r="K38" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L38" s="16" t="s">
+      <c r="L38" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M38" s="16" t="s">
+      <c r="M38" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="N38" s="16" t="s">
+      <c r="N38" s="18" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A39" s="20"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="20"/>
+      <c r="A39" s="19"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
       <c r="F39" s="2" t="s">
         <v>173</v>
       </c>
@@ -3764,12 +3637,12 @@
         <v>174</v>
       </c>
       <c r="H39" s="2"/>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20"/>
-      <c r="L39" s="20"/>
-      <c r="M39" s="20"/>
-      <c r="N39" s="20"/>
+      <c r="I39" s="19"/>
+      <c r="J39" s="19"/>
+      <c r="K39" s="19"/>
+      <c r="L39" s="19"/>
+      <c r="M39" s="19"/>
+      <c r="N39" s="19"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A40" s="17"/>
@@ -3792,19 +3665,19 @@
       <c r="N40" s="17"/>
     </row>
     <row r="41" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="26" t="s">
+      <c r="A41" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B41" s="18" t="s">
+      <c r="B41" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="C41" s="16" t="s">
+      <c r="C41" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="D41" s="16" t="s">
+      <c r="D41" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="E41" s="16" t="s">
+      <c r="E41" s="18" t="s">
         <v>179</v>
       </c>
       <c r="F41" s="2" t="s">
@@ -3816,22 +3689,22 @@
       <c r="H41" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="I41" s="16" t="s">
+      <c r="I41" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J41" s="16" t="s">
+      <c r="J41" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K41" s="16" t="s">
+      <c r="K41" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L41" s="16" t="s">
+      <c r="L41" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M41" s="16" t="s">
+      <c r="M41" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="N41" s="16" t="s">
+      <c r="N41" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3856,19 +3729,19 @@
       <c r="N42" s="17"/>
     </row>
     <row r="43" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A43" s="22" t="s">
+      <c r="A43" s="26" t="s">
         <v>185</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="C43" s="16" t="s">
+      <c r="C43" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="D43" s="16" t="s">
+      <c r="D43" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="E43" s="16" t="s">
+      <c r="E43" s="18" t="s">
         <v>189</v>
       </c>
       <c r="F43" s="2" t="s">
@@ -3880,22 +3753,22 @@
       <c r="H43" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="I43" s="16" t="s">
+      <c r="I43" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J43" s="16" t="s">
+      <c r="J43" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K43" s="16" t="s">
+      <c r="K43" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L43" s="16" t="s">
+      <c r="L43" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M43" s="16" t="s">
+      <c r="M43" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="N43" s="16" t="s">
+      <c r="N43" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3920,19 +3793,19 @@
       <c r="N44" s="17"/>
     </row>
     <row r="45" spans="1:14" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A45" s="22" t="s">
+      <c r="A45" s="26" t="s">
         <v>185</v>
       </c>
-      <c r="B45" s="18" t="s">
+      <c r="B45" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C45" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="D45" s="16" t="s">
+      <c r="D45" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="E45" s="16" t="s">
+      <c r="E45" s="18" t="s">
         <v>197</v>
       </c>
       <c r="F45" s="2" t="s">
@@ -3944,22 +3817,22 @@
       <c r="H45" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="I45" s="16" t="s">
+      <c r="I45" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J45" s="16" t="s">
+      <c r="J45" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K45" s="16" t="s">
+      <c r="K45" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L45" s="16" t="s">
+      <c r="L45" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M45" s="16" t="s">
+      <c r="M45" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="N45" s="16" t="s">
+      <c r="N45" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3984,19 +3857,19 @@
       <c r="N46" s="17"/>
     </row>
     <row r="47" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A47" s="22" t="s">
+      <c r="A47" s="26" t="s">
         <v>185</v>
       </c>
-      <c r="B47" s="18" t="s">
+      <c r="B47" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="C47" s="16" t="s">
+      <c r="C47" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="D47" s="16" t="s">
+      <c r="D47" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="E47" s="16" t="s">
+      <c r="E47" s="18" t="s">
         <v>206</v>
       </c>
       <c r="F47" s="2" t="s">
@@ -4008,31 +3881,31 @@
       <c r="H47" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="I47" s="16" t="s">
+      <c r="I47" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J47" s="16" t="s">
+      <c r="J47" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K47" s="16" t="s">
+      <c r="K47" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L47" s="16" t="s">
+      <c r="L47" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M47" s="16" t="s">
+      <c r="M47" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="N47" s="16" t="s">
+      <c r="N47" s="18" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
+      <c r="A48" s="19"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
       <c r="F48" s="2" t="s">
         <v>210</v>
       </c>
@@ -4040,12 +3913,12 @@
         <v>211</v>
       </c>
       <c r="H48" s="2"/>
-      <c r="I48" s="20"/>
-      <c r="J48" s="20"/>
-      <c r="K48" s="20"/>
-      <c r="L48" s="20"/>
-      <c r="M48" s="20"/>
-      <c r="N48" s="20"/>
+      <c r="I48" s="19"/>
+      <c r="J48" s="19"/>
+      <c r="K48" s="19"/>
+      <c r="L48" s="19"/>
+      <c r="M48" s="19"/>
+      <c r="N48" s="19"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A49" s="17"/>
@@ -4068,19 +3941,19 @@
       <c r="N49" s="17"/>
     </row>
     <row r="50" spans="1:14" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="A50" s="22" t="s">
+      <c r="A50" s="26" t="s">
         <v>185</v>
       </c>
-      <c r="B50" s="18" t="s">
+      <c r="B50" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C50" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="D50" s="16" t="s">
+      <c r="D50" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="E50" s="16" t="s">
+      <c r="E50" s="18" t="s">
         <v>216</v>
       </c>
       <c r="F50" s="2" t="s">
@@ -4092,22 +3965,22 @@
       <c r="H50" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="I50" s="16" t="s">
+      <c r="I50" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J50" s="16" t="s">
+      <c r="J50" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K50" s="16" t="s">
+      <c r="K50" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L50" s="16" t="s">
+      <c r="L50" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M50" s="16" t="s">
+      <c r="M50" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="N50" s="16" t="s">
+      <c r="N50" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4132,19 +4005,19 @@
       <c r="N51" s="17"/>
     </row>
     <row r="52" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A52" s="27" t="s">
+      <c r="A52" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="B52" s="18" t="s">
+      <c r="B52" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="C52" s="16" t="s">
+      <c r="C52" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="D52" s="16" t="s">
+      <c r="D52" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="E52" s="16" t="s">
+      <c r="E52" s="18" t="s">
         <v>227</v>
       </c>
       <c r="F52" s="2" t="s">
@@ -4156,22 +4029,22 @@
       <c r="H52" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="I52" s="16" t="s">
+      <c r="I52" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J52" s="16" t="s">
+      <c r="J52" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K52" s="16" t="s">
+      <c r="K52" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L52" s="16" t="s">
+      <c r="L52" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M52" s="16" t="s">
+      <c r="M52" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="N52" s="16" t="s">
+      <c r="N52" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4196,19 +4069,19 @@
       <c r="N53" s="17"/>
     </row>
     <row r="54" spans="1:14" ht="87" x14ac:dyDescent="0.35">
-      <c r="A54" s="27" t="s">
+      <c r="A54" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="B54" s="18" t="s">
+      <c r="B54" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="C54" s="16" t="s">
+      <c r="C54" s="18" t="s">
         <v>234</v>
       </c>
-      <c r="D54" s="16" t="s">
+      <c r="D54" s="18" t="s">
         <v>235</v>
       </c>
-      <c r="E54" s="16" t="s">
+      <c r="E54" s="18" t="s">
         <v>236</v>
       </c>
       <c r="F54" s="2" t="s">
@@ -4220,22 +4093,22 @@
       <c r="H54" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="I54" s="16" t="s">
+      <c r="I54" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J54" s="16" t="s">
+      <c r="J54" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K54" s="16" t="s">
+      <c r="K54" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L54" s="16" t="s">
+      <c r="L54" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M54" s="16" t="s">
+      <c r="M54" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="N54" s="16" t="s">
+      <c r="N54" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4260,19 +4133,19 @@
       <c r="N55" s="17"/>
     </row>
     <row r="56" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="27" t="s">
+      <c r="A56" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="B56" s="18" t="s">
+      <c r="B56" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="C56" s="16" t="s">
+      <c r="C56" s="18" t="s">
         <v>242</v>
       </c>
-      <c r="D56" s="16" t="s">
+      <c r="D56" s="18" t="s">
         <v>243</v>
       </c>
-      <c r="E56" s="16" t="s">
+      <c r="E56" s="18" t="s">
         <v>244</v>
       </c>
       <c r="F56" s="2" t="s">
@@ -4284,22 +4157,22 @@
       <c r="H56" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="I56" s="16" t="s">
+      <c r="I56" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J56" s="16" t="s">
+      <c r="J56" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="K56" s="16" t="s">
+      <c r="K56" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L56" s="16" t="s">
+      <c r="L56" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M56" s="16" t="s">
+      <c r="M56" s="18" t="s">
         <v>249</v>
       </c>
-      <c r="N56" s="16" t="s">
+      <c r="N56" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4324,19 +4197,19 @@
       <c r="N57" s="17"/>
     </row>
     <row r="58" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="27" t="s">
+      <c r="A58" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="B58" s="18" t="s">
+      <c r="B58" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="C58" s="16" t="s">
+      <c r="C58" s="18" t="s">
         <v>252</v>
       </c>
-      <c r="D58" s="16" t="s">
+      <c r="D58" s="18" t="s">
         <v>253</v>
       </c>
-      <c r="E58" s="16" t="s">
+      <c r="E58" s="18" t="s">
         <v>254</v>
       </c>
       <c r="F58" s="2" t="s">
@@ -4348,22 +4221,22 @@
       <c r="H58" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="I58" s="16" t="s">
+      <c r="I58" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J58" s="16" t="s">
+      <c r="J58" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="K58" s="16" t="s">
+      <c r="K58" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L58" s="16" t="s">
+      <c r="L58" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M58" s="16" t="s">
+      <c r="M58" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="N58" s="16" t="s">
+      <c r="N58" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4388,19 +4261,19 @@
       <c r="N59" s="17"/>
     </row>
     <row r="60" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A60" s="28" t="s">
+      <c r="A60" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="B60" s="18" t="s">
+      <c r="B60" s="16" t="s">
         <v>261</v>
       </c>
-      <c r="C60" s="16" t="s">
+      <c r="C60" s="18" t="s">
         <v>262</v>
       </c>
-      <c r="D60" s="16" t="s">
+      <c r="D60" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="E60" s="16" t="s">
+      <c r="E60" s="18" t="s">
         <v>264</v>
       </c>
       <c r="F60" s="2" t="s">
@@ -4410,22 +4283,22 @@
         <v>266</v>
       </c>
       <c r="H60" s="2"/>
-      <c r="I60" s="16" t="s">
+      <c r="I60" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J60" s="16" t="s">
+      <c r="J60" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K60" s="16" t="s">
+      <c r="K60" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L60" s="16" t="s">
+      <c r="L60" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M60" s="16" t="s">
+      <c r="M60" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="N60" s="16" t="s">
+      <c r="N60" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4450,19 +4323,19 @@
       <c r="N61" s="17"/>
     </row>
     <row r="62" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A62" s="28" t="s">
+      <c r="A62" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="B62" s="18" t="s">
+      <c r="B62" s="16" t="s">
         <v>261</v>
       </c>
-      <c r="C62" s="16" t="s">
+      <c r="C62" s="18" t="s">
         <v>269</v>
       </c>
-      <c r="D62" s="16" t="s">
+      <c r="D62" s="18" t="s">
         <v>270</v>
       </c>
-      <c r="E62" s="16" t="s">
+      <c r="E62" s="18" t="s">
         <v>271</v>
       </c>
       <c r="F62" s="2" t="s">
@@ -4472,31 +4345,31 @@
         <v>273</v>
       </c>
       <c r="H62" s="2"/>
-      <c r="I62" s="16" t="s">
+      <c r="I62" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J62" s="16" t="s">
+      <c r="J62" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K62" s="16" t="s">
+      <c r="K62" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="L62" s="16" t="s">
+      <c r="L62" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M62" s="16" t="s">
+      <c r="M62" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="N62" s="16" t="s">
+      <c r="N62" s="18" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="63" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A63" s="20"/>
-      <c r="B63" s="20"/>
-      <c r="C63" s="20"/>
-      <c r="D63" s="20"/>
-      <c r="E63" s="20"/>
+      <c r="A63" s="19"/>
+      <c r="B63" s="19"/>
+      <c r="C63" s="19"/>
+      <c r="D63" s="19"/>
+      <c r="E63" s="19"/>
       <c r="F63" s="2" t="s">
         <v>274</v>
       </c>
@@ -4504,12 +4377,12 @@
         <v>275</v>
       </c>
       <c r="H63" s="2"/>
-      <c r="I63" s="20"/>
-      <c r="J63" s="20"/>
-      <c r="K63" s="20"/>
-      <c r="L63" s="20"/>
-      <c r="M63" s="20"/>
-      <c r="N63" s="20"/>
+      <c r="I63" s="19"/>
+      <c r="J63" s="19"/>
+      <c r="K63" s="19"/>
+      <c r="L63" s="19"/>
+      <c r="M63" s="19"/>
+      <c r="N63" s="19"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A64" s="17"/>
@@ -4532,19 +4405,19 @@
       <c r="N64" s="17"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A65" s="28" t="s">
+      <c r="A65" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="B65" s="18" t="s">
+      <c r="B65" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="C65" s="16" t="s">
+      <c r="C65" s="18" t="s">
         <v>279</v>
       </c>
-      <c r="D65" s="16" t="s">
+      <c r="D65" s="18" t="s">
         <v>280</v>
       </c>
-      <c r="E65" s="16" t="s">
+      <c r="E65" s="18" t="s">
         <v>281</v>
       </c>
       <c r="F65" s="2" t="s">
@@ -4554,31 +4427,31 @@
         <v>283</v>
       </c>
       <c r="H65" s="2"/>
-      <c r="I65" s="16" t="s">
+      <c r="I65" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J65" s="16" t="s">
+      <c r="J65" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K65" s="16" t="s">
+      <c r="K65" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="L65" s="16" t="s">
+      <c r="L65" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M65" s="16" t="s">
+      <c r="M65" s="18" t="s">
         <v>284</v>
       </c>
-      <c r="N65" s="16" t="s">
+      <c r="N65" s="18" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="66" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A66" s="20"/>
-      <c r="B66" s="20"/>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
-      <c r="E66" s="20"/>
+      <c r="A66" s="19"/>
+      <c r="B66" s="19"/>
+      <c r="C66" s="19"/>
+      <c r="D66" s="19"/>
+      <c r="E66" s="19"/>
       <c r="F66" s="2" t="s">
         <v>285</v>
       </c>
@@ -4586,12 +4459,12 @@
         <v>286</v>
       </c>
       <c r="H66" s="2"/>
-      <c r="I66" s="20"/>
-      <c r="J66" s="20"/>
-      <c r="K66" s="20"/>
-      <c r="L66" s="20"/>
-      <c r="M66" s="20"/>
-      <c r="N66" s="20"/>
+      <c r="I66" s="19"/>
+      <c r="J66" s="19"/>
+      <c r="K66" s="19"/>
+      <c r="L66" s="19"/>
+      <c r="M66" s="19"/>
+      <c r="N66" s="19"/>
     </row>
     <row r="67" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A67" s="17"/>
@@ -4614,19 +4487,19 @@
       <c r="N67" s="17"/>
     </row>
     <row r="68" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="28" t="s">
+      <c r="A68" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="B68" s="18" t="s">
+      <c r="B68" s="16" t="s">
         <v>289</v>
       </c>
-      <c r="C68" s="16" t="s">
+      <c r="C68" s="18" t="s">
         <v>290</v>
       </c>
-      <c r="D68" s="16" t="s">
+      <c r="D68" s="18" t="s">
         <v>291</v>
       </c>
-      <c r="E68" s="16" t="s">
+      <c r="E68" s="18" t="s">
         <v>292</v>
       </c>
       <c r="F68" s="2" t="s">
@@ -4636,31 +4509,31 @@
         <v>294</v>
       </c>
       <c r="H68" s="2"/>
-      <c r="I68" s="16" t="s">
+      <c r="I68" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J68" s="16" t="s">
+      <c r="J68" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K68" s="16" t="s">
+      <c r="K68" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L68" s="16" t="s">
+      <c r="L68" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M68" s="16" t="s">
+      <c r="M68" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="N68" s="16" t="s">
+      <c r="N68" s="18" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="69" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A69" s="20"/>
-      <c r="B69" s="20"/>
-      <c r="C69" s="20"/>
-      <c r="D69" s="20"/>
-      <c r="E69" s="20"/>
+      <c r="A69" s="19"/>
+      <c r="B69" s="19"/>
+      <c r="C69" s="19"/>
+      <c r="D69" s="19"/>
+      <c r="E69" s="19"/>
       <c r="F69" s="2" t="s">
         <v>295</v>
       </c>
@@ -4668,12 +4541,12 @@
         <v>296</v>
       </c>
       <c r="H69" s="2"/>
-      <c r="I69" s="20"/>
-      <c r="J69" s="20"/>
-      <c r="K69" s="20"/>
-      <c r="L69" s="20"/>
-      <c r="M69" s="20"/>
-      <c r="N69" s="20"/>
+      <c r="I69" s="19"/>
+      <c r="J69" s="19"/>
+      <c r="K69" s="19"/>
+      <c r="L69" s="19"/>
+      <c r="M69" s="19"/>
+      <c r="N69" s="19"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A70" s="17"/>
@@ -4696,19 +4569,19 @@
       <c r="N70" s="17"/>
     </row>
     <row r="71" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A71" s="28" t="s">
+      <c r="A71" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="B71" s="18" t="s">
+      <c r="B71" s="16" t="s">
         <v>299</v>
       </c>
-      <c r="C71" s="16" t="s">
+      <c r="C71" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="D71" s="16" t="s">
+      <c r="D71" s="18" t="s">
         <v>301</v>
       </c>
-      <c r="E71" s="16" t="s">
+      <c r="E71" s="18" t="s">
         <v>302</v>
       </c>
       <c r="F71" s="2" t="s">
@@ -4718,22 +4591,22 @@
         <v>304</v>
       </c>
       <c r="H71" s="2"/>
-      <c r="I71" s="16" t="s">
+      <c r="I71" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J71" s="16" t="s">
+      <c r="J71" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K71" s="16" t="s">
+      <c r="K71" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L71" s="16" t="s">
+      <c r="L71" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M71" s="16" t="s">
+      <c r="M71" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="N71" s="16" t="s">
+      <c r="N71" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4758,19 +4631,19 @@
       <c r="N72" s="17"/>
     </row>
     <row r="73" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="28" t="s">
+      <c r="A73" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="B73" s="18" t="s">
+      <c r="B73" s="16" t="s">
         <v>307</v>
       </c>
-      <c r="C73" s="16" t="s">
+      <c r="C73" s="18" t="s">
         <v>308</v>
       </c>
-      <c r="D73" s="16" t="s">
+      <c r="D73" s="18" t="s">
         <v>309</v>
       </c>
-      <c r="E73" s="16" t="s">
+      <c r="E73" s="18" t="s">
         <v>310</v>
       </c>
       <c r="F73" s="2" t="s">
@@ -4780,22 +4653,22 @@
         <v>312</v>
       </c>
       <c r="H73" s="2"/>
-      <c r="I73" s="16" t="s">
+      <c r="I73" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J73" s="16" t="s">
+      <c r="J73" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K73" s="16" t="s">
+      <c r="K73" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L73" s="16" t="s">
+      <c r="L73" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M73" s="16" t="s">
+      <c r="M73" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="N73" s="16" t="s">
+      <c r="N73" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4820,19 +4693,19 @@
       <c r="N74" s="17"/>
     </row>
     <row r="75" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A75" s="21" t="s">
+      <c r="A75" s="25" t="s">
         <v>315</v>
       </c>
-      <c r="B75" s="18" t="s">
+      <c r="B75" s="16" t="s">
         <v>316</v>
       </c>
-      <c r="C75" s="16" t="s">
+      <c r="C75" s="18" t="s">
         <v>317</v>
       </c>
-      <c r="D75" s="16" t="s">
+      <c r="D75" s="18" t="s">
         <v>318</v>
       </c>
-      <c r="E75" s="16" t="s">
+      <c r="E75" s="18" t="s">
         <v>319</v>
       </c>
       <c r="F75" s="2" t="s">
@@ -4842,22 +4715,22 @@
         <v>321</v>
       </c>
       <c r="H75" s="2"/>
-      <c r="I75" s="16" t="s">
+      <c r="I75" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J75" s="16" t="s">
+      <c r="J75" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K75" s="16" t="s">
+      <c r="K75" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L75" s="16" t="s">
+      <c r="L75" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M75" s="16" t="s">
+      <c r="M75" s="18" t="s">
         <v>322</v>
       </c>
-      <c r="N75" s="16" t="s">
+      <c r="N75" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4882,19 +4755,19 @@
       <c r="N76" s="17"/>
     </row>
     <row r="77" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A77" s="21" t="s">
+      <c r="A77" s="25" t="s">
         <v>315</v>
       </c>
-      <c r="B77" s="18" t="s">
+      <c r="B77" s="16" t="s">
         <v>316</v>
       </c>
-      <c r="C77" s="16" t="s">
+      <c r="C77" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="D77" s="16" t="s">
+      <c r="D77" s="18" t="s">
         <v>326</v>
       </c>
-      <c r="E77" s="16" t="s">
+      <c r="E77" s="18" t="s">
         <v>327</v>
       </c>
       <c r="F77" s="2" t="s">
@@ -4904,22 +4777,22 @@
         <v>329</v>
       </c>
       <c r="H77" s="2"/>
-      <c r="I77" s="16" t="s">
+      <c r="I77" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J77" s="16" t="s">
+      <c r="J77" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K77" s="16" t="s">
+      <c r="K77" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L77" s="16" t="s">
+      <c r="L77" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M77" s="16" t="s">
+      <c r="M77" s="18" t="s">
         <v>322</v>
       </c>
-      <c r="N77" s="16" t="s">
+      <c r="N77" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4944,19 +4817,19 @@
       <c r="N78" s="17"/>
     </row>
     <row r="79" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="21" t="s">
+      <c r="A79" s="25" t="s">
         <v>315</v>
       </c>
-      <c r="B79" s="18" t="s">
+      <c r="B79" s="16" t="s">
         <v>316</v>
       </c>
-      <c r="C79" s="16" t="s">
+      <c r="C79" s="18" t="s">
         <v>332</v>
       </c>
-      <c r="D79" s="16" t="s">
+      <c r="D79" s="18" t="s">
         <v>333</v>
       </c>
-      <c r="E79" s="16" t="s">
+      <c r="E79" s="18" t="s">
         <v>334</v>
       </c>
       <c r="F79" s="2" t="s">
@@ -4966,22 +4839,22 @@
         <v>336</v>
       </c>
       <c r="H79" s="2"/>
-      <c r="I79" s="16" t="s">
+      <c r="I79" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J79" s="16" t="s">
+      <c r="J79" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K79" s="16" t="s">
+      <c r="K79" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L79" s="16" t="s">
+      <c r="L79" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M79" s="16" t="s">
+      <c r="M79" s="18" t="s">
         <v>322</v>
       </c>
-      <c r="N79" s="16" t="s">
+      <c r="N79" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -5006,19 +4879,19 @@
       <c r="N80" s="17"/>
     </row>
     <row r="81" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="21" t="s">
+      <c r="A81" s="25" t="s">
         <v>315</v>
       </c>
-      <c r="B81" s="18" t="s">
+      <c r="B81" s="16" t="s">
         <v>316</v>
       </c>
-      <c r="C81" s="16" t="s">
+      <c r="C81" s="18" t="s">
         <v>339</v>
       </c>
-      <c r="D81" s="16" t="s">
+      <c r="D81" s="18" t="s">
         <v>340</v>
       </c>
-      <c r="E81" s="16" t="s">
+      <c r="E81" s="18" t="s">
         <v>341</v>
       </c>
       <c r="F81" s="2" t="s">
@@ -5028,22 +4901,22 @@
         <v>343</v>
       </c>
       <c r="H81" s="2"/>
-      <c r="I81" s="16" t="s">
+      <c r="I81" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J81" s="16" t="s">
+      <c r="J81" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K81" s="16" t="s">
+      <c r="K81" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L81" s="16" t="s">
+      <c r="L81" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M81" s="16" t="s">
+      <c r="M81" s="18" t="s">
         <v>322</v>
       </c>
-      <c r="N81" s="16" t="s">
+      <c r="N81" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -5068,19 +4941,19 @@
       <c r="N82" s="17"/>
     </row>
     <row r="83" spans="1:14" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="A83" s="23" t="s">
+      <c r="A83" s="21" t="s">
         <v>346</v>
       </c>
-      <c r="B83" s="18" t="s">
+      <c r="B83" s="16" t="s">
         <v>347</v>
       </c>
-      <c r="C83" s="16" t="s">
+      <c r="C83" s="18" t="s">
         <v>348</v>
       </c>
-      <c r="D83" s="16" t="s">
+      <c r="D83" s="18" t="s">
         <v>349</v>
       </c>
-      <c r="E83" s="16" t="s">
+      <c r="E83" s="18" t="s">
         <v>350</v>
       </c>
       <c r="F83" s="2" t="s">
@@ -5092,22 +4965,22 @@
       <c r="H83" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="I83" s="16" t="s">
+      <c r="I83" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J83" s="16" t="s">
+      <c r="J83" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K83" s="16" t="s">
+      <c r="K83" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L83" s="16" t="s">
+      <c r="L83" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M83" s="16" t="s">
+      <c r="M83" s="18" t="s">
         <v>354</v>
       </c>
-      <c r="N83" s="16" t="s">
+      <c r="N83" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -5132,19 +5005,19 @@
       <c r="N84" s="17"/>
     </row>
     <row r="85" spans="1:14" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="A85" s="23" t="s">
+      <c r="A85" s="21" t="s">
         <v>346</v>
       </c>
-      <c r="B85" s="18" t="s">
+      <c r="B85" s="16" t="s">
         <v>357</v>
       </c>
-      <c r="C85" s="16" t="s">
+      <c r="C85" s="18" t="s">
         <v>358</v>
       </c>
-      <c r="D85" s="16" t="s">
+      <c r="D85" s="18" t="s">
         <v>359</v>
       </c>
-      <c r="E85" s="16" t="s">
+      <c r="E85" s="18" t="s">
         <v>360</v>
       </c>
       <c r="F85" s="2" t="s">
@@ -5156,22 +5029,22 @@
       <c r="H85" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="I85" s="16" t="s">
+      <c r="I85" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J85" s="16" t="s">
+      <c r="J85" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K85" s="16" t="s">
+      <c r="K85" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L85" s="16" t="s">
+      <c r="L85" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M85" s="16" t="s">
+      <c r="M85" s="18" t="s">
         <v>364</v>
       </c>
-      <c r="N85" s="16" t="s">
+      <c r="N85" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -5196,19 +5069,19 @@
       <c r="N86" s="17"/>
     </row>
     <row r="87" spans="1:14" ht="217.5" x14ac:dyDescent="0.35">
-      <c r="A87" s="23" t="s">
+      <c r="A87" s="21" t="s">
         <v>346</v>
       </c>
-      <c r="B87" s="18" t="s">
+      <c r="B87" s="16" t="s">
         <v>357</v>
       </c>
-      <c r="C87" s="16" t="s">
+      <c r="C87" s="18" t="s">
         <v>367</v>
       </c>
-      <c r="D87" s="16" t="s">
+      <c r="D87" s="18" t="s">
         <v>368</v>
       </c>
-      <c r="E87" s="16" t="s">
+      <c r="E87" s="18" t="s">
         <v>369</v>
       </c>
       <c r="F87" s="2" t="s">
@@ -5220,22 +5093,22 @@
       <c r="H87" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="I87" s="16" t="s">
+      <c r="I87" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J87" s="16" t="s">
+      <c r="J87" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="K87" s="16" t="s">
+      <c r="K87" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L87" s="16" t="s">
+      <c r="L87" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M87" s="16" t="s">
+      <c r="M87" s="18" t="s">
         <v>373</v>
       </c>
-      <c r="N87" s="16" t="s">
+      <c r="N87" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -5260,19 +5133,19 @@
       <c r="N88" s="17"/>
     </row>
     <row r="89" spans="1:14" ht="362.5" x14ac:dyDescent="0.35">
-      <c r="A89" s="24" t="s">
+      <c r="A89" s="27" t="s">
         <v>376</v>
       </c>
-      <c r="B89" s="18" t="s">
+      <c r="B89" s="16" t="s">
         <v>377</v>
       </c>
-      <c r="C89" s="16" t="s">
+      <c r="C89" s="18" t="s">
         <v>378</v>
       </c>
-      <c r="D89" s="16" t="s">
+      <c r="D89" s="18" t="s">
         <v>379</v>
       </c>
-      <c r="E89" s="16" t="s">
+      <c r="E89" s="18" t="s">
         <v>380</v>
       </c>
       <c r="F89" s="2" t="s">
@@ -5284,22 +5157,22 @@
       <c r="H89" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="I89" s="16" t="s">
+      <c r="I89" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J89" s="16" t="s">
+      <c r="J89" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K89" s="16" t="s">
+      <c r="K89" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L89" s="16" t="s">
+      <c r="L89" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M89" s="16" t="s">
+      <c r="M89" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="N89" s="16" t="s">
+      <c r="N89" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -5324,19 +5197,19 @@
       <c r="N90" s="17"/>
     </row>
     <row r="91" spans="1:14" ht="217.5" x14ac:dyDescent="0.35">
-      <c r="A91" s="24" t="s">
+      <c r="A91" s="27" t="s">
         <v>376</v>
       </c>
-      <c r="B91" s="18" t="s">
+      <c r="B91" s="16" t="s">
         <v>377</v>
       </c>
-      <c r="C91" s="16" t="s">
+      <c r="C91" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="D91" s="16" t="s">
+      <c r="D91" s="18" t="s">
         <v>388</v>
       </c>
-      <c r="E91" s="16" t="s">
+      <c r="E91" s="18" t="s">
         <v>389</v>
       </c>
       <c r="F91" s="2" t="s">
@@ -5348,22 +5221,22 @@
       <c r="H91" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="I91" s="16" t="s">
+      <c r="I91" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J91" s="16" t="s">
+      <c r="J91" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K91" s="16" t="s">
+      <c r="K91" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L91" s="16" t="s">
+      <c r="L91" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M91" s="16" t="s">
+      <c r="M91" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="N91" s="16" t="s">
+      <c r="N91" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -5388,19 +5261,19 @@
       <c r="N92" s="17"/>
     </row>
     <row r="93" spans="1:14" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A93" s="24" t="s">
+      <c r="A93" s="27" t="s">
         <v>395</v>
       </c>
-      <c r="B93" s="18" t="s">
+      <c r="B93" s="16" t="s">
         <v>396</v>
       </c>
-      <c r="C93" s="16" t="s">
+      <c r="C93" s="18" t="s">
         <v>397</v>
       </c>
-      <c r="D93" s="16" t="s">
+      <c r="D93" s="18" t="s">
         <v>398</v>
       </c>
-      <c r="E93" s="16" t="s">
+      <c r="E93" s="18" t="s">
         <v>399</v>
       </c>
       <c r="F93" s="2" t="s">
@@ -5412,22 +5285,22 @@
       <c r="H93" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="I93" s="16" t="s">
-        <v>629</v>
-      </c>
-      <c r="J93" s="16" t="s">
+      <c r="I93" s="18" t="s">
+        <v>587</v>
+      </c>
+      <c r="J93" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K93" s="16" t="s">
+      <c r="K93" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L93" s="16" t="s">
+      <c r="L93" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M93" s="16" t="s">
+      <c r="M93" s="18" t="s">
         <v>403</v>
       </c>
-      <c r="N93" s="16" t="s">
+      <c r="N93" s="18" t="s">
         <v>404</v>
       </c>
     </row>
@@ -5452,19 +5325,19 @@
       <c r="N94" s="17"/>
     </row>
     <row r="95" spans="1:14" ht="275.5" x14ac:dyDescent="0.35">
-      <c r="A95" s="24" t="s">
+      <c r="A95" s="27" t="s">
         <v>395</v>
       </c>
-      <c r="B95" s="18" t="s">
+      <c r="B95" s="16" t="s">
         <v>407</v>
       </c>
-      <c r="C95" s="16" t="s">
+      <c r="C95" s="18" t="s">
         <v>408</v>
       </c>
-      <c r="D95" s="16" t="s">
+      <c r="D95" s="18" t="s">
         <v>409</v>
       </c>
-      <c r="E95" s="16" t="s">
+      <c r="E95" s="18" t="s">
         <v>410</v>
       </c>
       <c r="F95" s="2" t="s">
@@ -5476,22 +5349,22 @@
       <c r="H95" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="I95" s="16" t="s">
-        <v>629</v>
-      </c>
-      <c r="J95" s="16" t="s">
+      <c r="I95" s="18" t="s">
+        <v>587</v>
+      </c>
+      <c r="J95" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K95" s="16" t="s">
+      <c r="K95" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L95" s="16" t="s">
+      <c r="L95" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M95" s="16" t="s">
+      <c r="M95" s="18" t="s">
         <v>403</v>
       </c>
-      <c r="N95" s="16" t="s">
+      <c r="N95" s="18" t="s">
         <v>404</v>
       </c>
     </row>
@@ -5516,19 +5389,19 @@
       <c r="N96" s="17"/>
     </row>
     <row r="97" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A97" s="19" t="s">
+      <c r="A97" s="28" t="s">
         <v>416</v>
       </c>
-      <c r="B97" s="18" t="s">
+      <c r="B97" s="16" t="s">
         <v>417</v>
       </c>
-      <c r="C97" s="16" t="s">
+      <c r="C97" s="18" t="s">
         <v>418</v>
       </c>
-      <c r="D97" s="16" t="s">
+      <c r="D97" s="18" t="s">
         <v>419</v>
       </c>
-      <c r="E97" s="16" t="s">
+      <c r="E97" s="18" t="s">
         <v>420</v>
       </c>
       <c r="F97" s="2" t="s">
@@ -5538,22 +5411,22 @@
         <v>422</v>
       </c>
       <c r="H97" s="2"/>
-      <c r="I97" s="16" t="s">
+      <c r="I97" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J97" s="16" t="s">
+      <c r="J97" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="K97" s="16" t="s">
+      <c r="K97" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L97" s="16" t="s">
+      <c r="L97" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M97" s="16" t="s">
+      <c r="M97" s="18" t="s">
         <v>423</v>
       </c>
-      <c r="N97" s="16" t="s">
+      <c r="N97" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -5578,19 +5451,19 @@
       <c r="N98" s="17"/>
     </row>
     <row r="99" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="19" t="s">
+      <c r="A99" s="28" t="s">
         <v>416</v>
       </c>
-      <c r="B99" s="18" t="s">
+      <c r="B99" s="16" t="s">
         <v>426</v>
       </c>
-      <c r="C99" s="16" t="s">
+      <c r="C99" s="18" t="s">
         <v>427</v>
       </c>
-      <c r="D99" s="16" t="s">
+      <c r="D99" s="18" t="s">
         <v>428</v>
       </c>
-      <c r="E99" s="16" t="s">
+      <c r="E99" s="18" t="s">
         <v>429</v>
       </c>
       <c r="F99" s="2" t="s">
@@ -5600,22 +5473,22 @@
         <v>431</v>
       </c>
       <c r="H99" s="2"/>
-      <c r="I99" s="16" t="s">
+      <c r="I99" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="J99" s="16" t="s">
+      <c r="J99" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="K99" s="16" t="s">
+      <c r="K99" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="L99" s="16" t="s">
+      <c r="L99" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="M99" s="16" t="s">
+      <c r="M99" s="18" t="s">
         <v>423</v>
       </c>
-      <c r="N99" s="16" t="s">
+      <c r="N99" s="18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -6191,15 +6064,464 @@
   </sheetData>
   <autoFilter ref="A1:N163" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="506">
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="I62:I64"/>
-    <mergeCell ref="C65:C67"/>
-    <mergeCell ref="N2:N4"/>
-    <mergeCell ref="N91:N92"/>
-    <mergeCell ref="A73:A74"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="D29:D31"/>
+    <mergeCell ref="D87:D88"/>
+    <mergeCell ref="I58:I59"/>
+    <mergeCell ref="K58:K59"/>
+    <mergeCell ref="K52:K53"/>
+    <mergeCell ref="J38:J40"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="I60:I61"/>
+    <mergeCell ref="J71:J72"/>
+    <mergeCell ref="J99:J100"/>
+    <mergeCell ref="E99:E100"/>
+    <mergeCell ref="D93:D94"/>
+    <mergeCell ref="A97:A98"/>
+    <mergeCell ref="D85:D86"/>
+    <mergeCell ref="I81:I82"/>
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="J77:J78"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="A87:A88"/>
+    <mergeCell ref="A89:A90"/>
+    <mergeCell ref="M91:M92"/>
+    <mergeCell ref="E91:E92"/>
+    <mergeCell ref="B95:B96"/>
+    <mergeCell ref="M41:M42"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="M93:M94"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="M43:M44"/>
+    <mergeCell ref="J95:J96"/>
+    <mergeCell ref="J89:J90"/>
+    <mergeCell ref="L89:L90"/>
+    <mergeCell ref="I32:I33"/>
+    <mergeCell ref="K32:K33"/>
+    <mergeCell ref="J60:J61"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="M54:M55"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="D77:D78"/>
+    <mergeCell ref="M47:M49"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="L43:L44"/>
+    <mergeCell ref="D75:D76"/>
+    <mergeCell ref="I71:I72"/>
+    <mergeCell ref="K71:K72"/>
+    <mergeCell ref="I65:I67"/>
+    <mergeCell ref="M29:M31"/>
+    <mergeCell ref="K65:K67"/>
+    <mergeCell ref="I73:I74"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E38:E40"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="J73:J74"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="N56:N57"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="J87:J88"/>
+    <mergeCell ref="L87:L88"/>
+    <mergeCell ref="E47:E49"/>
+    <mergeCell ref="M25:M26"/>
+    <mergeCell ref="C68:C70"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="I79:I80"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="D83:D84"/>
+    <mergeCell ref="K73:K74"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="L77:L78"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="N41:N42"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="E68:E70"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="K29:K31"/>
+    <mergeCell ref="K87:K88"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="I50:I51"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="I45:I46"/>
+    <mergeCell ref="I85:I86"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="D47:D49"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="D38:D40"/>
+    <mergeCell ref="N93:N94"/>
+    <mergeCell ref="I97:I98"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="C93:C94"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="A85:A86"/>
+    <mergeCell ref="J45:J46"/>
+    <mergeCell ref="K77:K78"/>
+    <mergeCell ref="L45:L46"/>
+    <mergeCell ref="J32:J33"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D91:D92"/>
+    <mergeCell ref="A95:A96"/>
+    <mergeCell ref="K95:K96"/>
+    <mergeCell ref="I89:I90"/>
+    <mergeCell ref="N29:N31"/>
+    <mergeCell ref="M87:M88"/>
+    <mergeCell ref="M56:M57"/>
+    <mergeCell ref="L75:L76"/>
+    <mergeCell ref="N75:N76"/>
+    <mergeCell ref="L38:L40"/>
+    <mergeCell ref="N38:N40"/>
+    <mergeCell ref="M34:M35"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="L34:L35"/>
+    <mergeCell ref="L47:L49"/>
+    <mergeCell ref="N47:N49"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="M75:M76"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="L41:L42"/>
+    <mergeCell ref="I47:I49"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="J68:J70"/>
+    <mergeCell ref="L68:L70"/>
+    <mergeCell ref="N68:N70"/>
+    <mergeCell ref="N25:N26"/>
+    <mergeCell ref="B68:B70"/>
+    <mergeCell ref="D68:D70"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="N79:N80"/>
+    <mergeCell ref="K83:K84"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="M83:M84"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="E58:E59"/>
+    <mergeCell ref="E65:E67"/>
+    <mergeCell ref="N81:N82"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E60:E61"/>
+    <mergeCell ref="K45:K46"/>
+    <mergeCell ref="L83:L84"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="E62:E64"/>
+    <mergeCell ref="M23:M24"/>
+    <mergeCell ref="N54:N55"/>
+    <mergeCell ref="L29:L31"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="N77:N78"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="N62:N64"/>
+    <mergeCell ref="N50:N51"/>
+    <mergeCell ref="M13:M14"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="M15:M16"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="N43:N44"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="K27:K28"/>
+    <mergeCell ref="N36:N37"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="D62:D64"/>
+    <mergeCell ref="I91:I92"/>
+    <mergeCell ref="K2:K4"/>
+    <mergeCell ref="K91:K92"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="K41:K42"/>
+    <mergeCell ref="N34:N35"/>
+    <mergeCell ref="K85:K86"/>
+    <mergeCell ref="J91:J92"/>
+    <mergeCell ref="L2:L4"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="L91:L92"/>
+    <mergeCell ref="N85:N86"/>
+    <mergeCell ref="K89:K90"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="M2:M4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="J2:J4"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="B91:B92"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="J93:J94"/>
+    <mergeCell ref="B93:B94"/>
+    <mergeCell ref="C95:C96"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="E95:E96"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J97:J98"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="L36:L37"/>
+    <mergeCell ref="K93:K94"/>
+    <mergeCell ref="I95:I96"/>
+    <mergeCell ref="L93:L94"/>
+    <mergeCell ref="E93:E94"/>
+    <mergeCell ref="B97:B98"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="M36:M37"/>
+    <mergeCell ref="J56:J57"/>
+    <mergeCell ref="L56:L57"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="L62:L64"/>
+    <mergeCell ref="J83:J84"/>
+    <mergeCell ref="E87:E88"/>
+    <mergeCell ref="E89:E90"/>
+    <mergeCell ref="D73:D74"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="K99:K100"/>
+    <mergeCell ref="M99:M100"/>
+    <mergeCell ref="C99:C100"/>
+    <mergeCell ref="J54:J55"/>
+    <mergeCell ref="K68:K70"/>
+    <mergeCell ref="L54:L55"/>
+    <mergeCell ref="M68:M70"/>
+    <mergeCell ref="L99:L100"/>
+    <mergeCell ref="D99:D100"/>
+    <mergeCell ref="A93:A94"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="J47:J49"/>
+    <mergeCell ref="K60:K61"/>
+    <mergeCell ref="M60:M61"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="A54:A55"/>
+    <mergeCell ref="I29:I31"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="I87:I88"/>
+    <mergeCell ref="L58:L59"/>
+    <mergeCell ref="L65:L67"/>
+    <mergeCell ref="I56:I57"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="K56:K57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="M38:M40"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="L71:L72"/>
+    <mergeCell ref="I75:I76"/>
+    <mergeCell ref="K75:K76"/>
+    <mergeCell ref="N65:N67"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="K62:K64"/>
+    <mergeCell ref="M62:M64"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="M45:M46"/>
+    <mergeCell ref="M32:M33"/>
+    <mergeCell ref="L60:L61"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="N60:N61"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="M58:M59"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D97:D98"/>
+    <mergeCell ref="I93:I94"/>
+    <mergeCell ref="N23:N24"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="N87:N88"/>
+    <mergeCell ref="M89:M90"/>
+    <mergeCell ref="L97:L98"/>
+    <mergeCell ref="N97:N98"/>
+    <mergeCell ref="B89:B90"/>
+    <mergeCell ref="D81:D82"/>
+    <mergeCell ref="I77:I78"/>
+    <mergeCell ref="E97:E98"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="D79:D80"/>
+    <mergeCell ref="M52:M53"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C91:C92"/>
+    <mergeCell ref="D95:D96"/>
+    <mergeCell ref="N58:N59"/>
+    <mergeCell ref="N52:N53"/>
+    <mergeCell ref="C62:C64"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="J85:J86"/>
+    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="M71:M72"/>
+    <mergeCell ref="K81:K82"/>
+    <mergeCell ref="M81:M82"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="L79:L80"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="L73:L74"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="J79:J80"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="N99:N100"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="M65:M67"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="M73:M74"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I38:I40"/>
+    <mergeCell ref="K38:K40"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="N21:N22"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="L81:L82"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="L95:L96"/>
+    <mergeCell ref="I99:I100"/>
+    <mergeCell ref="N95:N96"/>
+    <mergeCell ref="N89:N90"/>
+    <mergeCell ref="K79:K80"/>
+    <mergeCell ref="M79:M80"/>
+    <mergeCell ref="C97:C98"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="A68:A70"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="J36:J37"/>
+    <mergeCell ref="B62:B64"/>
+    <mergeCell ref="M17:M18"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="K47:K49"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="M50:M51"/>
+    <mergeCell ref="I68:I70"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="J34:J35"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="E54:E55"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="L32:L33"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="B65:B67"/>
+    <mergeCell ref="J62:J64"/>
+    <mergeCell ref="I36:I37"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A65:A67"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="I54:I55"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="M95:M96"/>
+    <mergeCell ref="J50:J51"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="N83:N84"/>
+    <mergeCell ref="L50:L51"/>
+    <mergeCell ref="N45:N46"/>
+    <mergeCell ref="N32:N33"/>
+    <mergeCell ref="K21:K22"/>
+    <mergeCell ref="D89:D90"/>
+    <mergeCell ref="I34:I35"/>
+    <mergeCell ref="K34:K35"/>
+    <mergeCell ref="C87:C88"/>
+    <mergeCell ref="I83:I84"/>
+    <mergeCell ref="N73:N74"/>
+    <mergeCell ref="L85:L86"/>
+    <mergeCell ref="N71:N72"/>
+    <mergeCell ref="K54:K55"/>
+    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="K43:K44"/>
+    <mergeCell ref="D71:D72"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D65:D67"/>
+    <mergeCell ref="J29:J31"/>
     <mergeCell ref="B99:B100"/>
     <mergeCell ref="E29:E31"/>
     <mergeCell ref="K97:K98"/>
@@ -6224,6 +6546,15 @@
     <mergeCell ref="J65:J67"/>
     <mergeCell ref="M85:M86"/>
     <mergeCell ref="E85:E86"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="I62:I64"/>
+    <mergeCell ref="C65:C67"/>
+    <mergeCell ref="N2:N4"/>
+    <mergeCell ref="N91:N92"/>
+    <mergeCell ref="A73:A74"/>
     <mergeCell ref="N17:N18"/>
     <mergeCell ref="C21:C22"/>
     <mergeCell ref="D41:D42"/>
@@ -6231,472 +6562,14 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D43:D44"/>
     <mergeCell ref="J75:J76"/>
-    <mergeCell ref="M95:M96"/>
-    <mergeCell ref="J50:J51"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="N83:N84"/>
-    <mergeCell ref="L50:L51"/>
-    <mergeCell ref="N45:N46"/>
-    <mergeCell ref="N32:N33"/>
-    <mergeCell ref="K21:K22"/>
-    <mergeCell ref="D89:D90"/>
     <mergeCell ref="I2:I4"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="A23:A24"/>
-    <mergeCell ref="I34:I35"/>
-    <mergeCell ref="K34:K35"/>
-    <mergeCell ref="C87:C88"/>
     <mergeCell ref="A52:A53"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="B38:B40"/>
     <mergeCell ref="K5:K6"/>
     <mergeCell ref="C5:C6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="B65:B67"/>
-    <mergeCell ref="J62:J64"/>
-    <mergeCell ref="I36:I37"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A65:A67"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="A68:A70"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="A71:A72"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="J36:J37"/>
-    <mergeCell ref="B62:B64"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="K47:K49"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="M50:M51"/>
-    <mergeCell ref="I68:I70"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="J34:J35"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="E54:E55"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="L32:L33"/>
-    <mergeCell ref="N99:N100"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="M65:M67"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="M73:M74"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I38:I40"/>
-    <mergeCell ref="K38:K40"/>
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="N21:N22"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="D45:D46"/>
-    <mergeCell ref="L81:L82"/>
-    <mergeCell ref="A77:A78"/>
-    <mergeCell ref="L95:L96"/>
-    <mergeCell ref="I99:I100"/>
-    <mergeCell ref="N95:N96"/>
-    <mergeCell ref="N89:N90"/>
-    <mergeCell ref="K79:K80"/>
-    <mergeCell ref="M79:M80"/>
-    <mergeCell ref="C97:C98"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="K13:K14"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="A81:A82"/>
-    <mergeCell ref="J41:J42"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="M71:M72"/>
-    <mergeCell ref="K81:K82"/>
-    <mergeCell ref="M81:M82"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="L79:L80"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="I83:I84"/>
-    <mergeCell ref="L73:L74"/>
-    <mergeCell ref="N73:N74"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="D97:D98"/>
-    <mergeCell ref="I93:I94"/>
-    <mergeCell ref="N23:N24"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="N87:N88"/>
-    <mergeCell ref="M89:M90"/>
-    <mergeCell ref="L97:L98"/>
-    <mergeCell ref="N97:N98"/>
-    <mergeCell ref="B89:B90"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="D81:D82"/>
-    <mergeCell ref="I77:I78"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="L71:L72"/>
-    <mergeCell ref="I75:I76"/>
-    <mergeCell ref="K75:K76"/>
-    <mergeCell ref="N65:N67"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="K62:K64"/>
-    <mergeCell ref="M62:M64"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="M45:M46"/>
-    <mergeCell ref="M32:M33"/>
-    <mergeCell ref="L60:L61"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="N60:N61"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="M58:M59"/>
-    <mergeCell ref="E97:E98"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="D79:D80"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="M52:M53"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C91:C92"/>
-    <mergeCell ref="A93:A94"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="J47:J49"/>
-    <mergeCell ref="K60:K61"/>
-    <mergeCell ref="M60:M61"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="A75:A76"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="D95:D96"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="A54:A55"/>
-    <mergeCell ref="I29:I31"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="I87:I88"/>
-    <mergeCell ref="L58:L59"/>
-    <mergeCell ref="L65:L67"/>
-    <mergeCell ref="N58:N59"/>
-    <mergeCell ref="I56:I57"/>
-    <mergeCell ref="N52:N53"/>
-    <mergeCell ref="A56:A57"/>
-    <mergeCell ref="K56:K57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="M38:M40"/>
-    <mergeCell ref="C62:C64"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="J85:J86"/>
-    <mergeCell ref="L85:L86"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="N71:N72"/>
-    <mergeCell ref="J79:J80"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="K25:K26"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="I54:I55"/>
-    <mergeCell ref="K54:K55"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="K43:K44"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="D71:D72"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="D65:D67"/>
-    <mergeCell ref="J29:J31"/>
-    <mergeCell ref="D73:D74"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="K99:K100"/>
-    <mergeCell ref="M99:M100"/>
-    <mergeCell ref="C99:C100"/>
-    <mergeCell ref="J54:J55"/>
-    <mergeCell ref="K68:K70"/>
-    <mergeCell ref="L54:L55"/>
-    <mergeCell ref="M68:M70"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="M36:M37"/>
-    <mergeCell ref="J56:J57"/>
-    <mergeCell ref="L56:L57"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="L62:L64"/>
-    <mergeCell ref="J83:J84"/>
-    <mergeCell ref="E87:E88"/>
-    <mergeCell ref="E89:E90"/>
-    <mergeCell ref="B91:B92"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="J93:J94"/>
-    <mergeCell ref="B93:B94"/>
-    <mergeCell ref="C95:C96"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="E95:E96"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="J97:J98"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="L36:L37"/>
-    <mergeCell ref="N36:N37"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="D62:D64"/>
-    <mergeCell ref="I91:I92"/>
-    <mergeCell ref="K2:K4"/>
-    <mergeCell ref="K91:K92"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="K41:K42"/>
-    <mergeCell ref="N34:N35"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="N77:N78"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="N62:N64"/>
-    <mergeCell ref="N50:N51"/>
-    <mergeCell ref="M13:M14"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="L99:L100"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="N79:N80"/>
-    <mergeCell ref="K83:K84"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="M83:M84"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="K93:K94"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="E58:E59"/>
-    <mergeCell ref="E65:E67"/>
-    <mergeCell ref="N81:N82"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="K85:K86"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E60:E61"/>
-    <mergeCell ref="K45:K46"/>
-    <mergeCell ref="M15:M16"/>
-    <mergeCell ref="J91:J92"/>
-    <mergeCell ref="L2:L4"/>
-    <mergeCell ref="N13:N14"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="L34:L35"/>
-    <mergeCell ref="L47:L49"/>
-    <mergeCell ref="N47:N49"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="M75:M76"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="L41:L42"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="I47:I49"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="B75:B76"/>
-    <mergeCell ref="J68:J70"/>
-    <mergeCell ref="L68:L70"/>
-    <mergeCell ref="N68:N70"/>
-    <mergeCell ref="L91:L92"/>
-    <mergeCell ref="I95:I96"/>
-    <mergeCell ref="D99:D100"/>
-    <mergeCell ref="N25:N26"/>
-    <mergeCell ref="N85:N86"/>
-    <mergeCell ref="B68:B70"/>
-    <mergeCell ref="K89:K90"/>
-    <mergeCell ref="D68:D70"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="L83:L84"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="L93:L94"/>
-    <mergeCell ref="N93:N94"/>
-    <mergeCell ref="I97:I98"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="C93:C94"/>
-    <mergeCell ref="A91:A92"/>
-    <mergeCell ref="A85:A86"/>
-    <mergeCell ref="J45:J46"/>
-    <mergeCell ref="K77:K78"/>
-    <mergeCell ref="L45:L46"/>
-    <mergeCell ref="J32:J33"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="D91:D92"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="A95:A96"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="E68:E70"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="K29:K31"/>
-    <mergeCell ref="K87:K88"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="I50:I51"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="K95:K96"/>
-    <mergeCell ref="I45:I46"/>
-    <mergeCell ref="I85:I86"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="D47:D49"/>
-    <mergeCell ref="I89:I90"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="N29:N31"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="D38:D40"/>
-    <mergeCell ref="M2:M4"/>
-    <mergeCell ref="M87:M88"/>
-    <mergeCell ref="M56:M57"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="L75:L76"/>
-    <mergeCell ref="N75:N76"/>
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="L38:L40"/>
-    <mergeCell ref="N38:N40"/>
-    <mergeCell ref="M34:M35"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="E62:E64"/>
-    <mergeCell ref="J2:J4"/>
-    <mergeCell ref="M23:M24"/>
-    <mergeCell ref="N54:N55"/>
-    <mergeCell ref="L29:L31"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="N56:N57"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="J87:J88"/>
-    <mergeCell ref="L87:L88"/>
-    <mergeCell ref="E47:E49"/>
-    <mergeCell ref="M25:M26"/>
-    <mergeCell ref="C68:C70"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="I79:I80"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="D83:D84"/>
-    <mergeCell ref="K73:K74"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="L77:L78"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="N41:N42"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="D77:D78"/>
-    <mergeCell ref="M47:M49"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="L43:L44"/>
-    <mergeCell ref="N43:N44"/>
-    <mergeCell ref="D75:D76"/>
-    <mergeCell ref="I71:I72"/>
-    <mergeCell ref="K71:K72"/>
-    <mergeCell ref="I65:I67"/>
-    <mergeCell ref="M29:M31"/>
-    <mergeCell ref="K65:K67"/>
-    <mergeCell ref="I73:I74"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E38:E40"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="J73:J74"/>
-    <mergeCell ref="E93:E94"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="B97:B98"/>
-    <mergeCell ref="A79:A80"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="J77:J78"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="A87:A88"/>
-    <mergeCell ref="A89:A90"/>
-    <mergeCell ref="M91:M92"/>
-    <mergeCell ref="E91:E92"/>
-    <mergeCell ref="B95:B96"/>
-    <mergeCell ref="M41:M42"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="M93:M94"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="M43:M44"/>
-    <mergeCell ref="J95:J96"/>
-    <mergeCell ref="J89:J90"/>
-    <mergeCell ref="L89:L90"/>
-    <mergeCell ref="I32:I33"/>
-    <mergeCell ref="K32:K33"/>
-    <mergeCell ref="J60:J61"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="M54:M55"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="K27:K28"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="D29:D31"/>
-    <mergeCell ref="D87:D88"/>
-    <mergeCell ref="I58:I59"/>
-    <mergeCell ref="K58:K59"/>
-    <mergeCell ref="K52:K53"/>
-    <mergeCell ref="J38:J40"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="I60:I61"/>
-    <mergeCell ref="J71:J72"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="J99:J100"/>
-    <mergeCell ref="E99:E100"/>
-    <mergeCell ref="D93:D94"/>
-    <mergeCell ref="A97:A98"/>
-    <mergeCell ref="D85:D86"/>
-    <mergeCell ref="I81:I82"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7295,188 +7168,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="70" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="9" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>587</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>588</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>589</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>592</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>595</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>596</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>597</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>600</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="D4" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>602</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>603</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="D5" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>605</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>607</v>
-      </c>
-      <c r="D6" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>608</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>609</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>612</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="D9" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>619</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>621</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>623</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="5" t="s">
-        <v>626</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>627</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>628</v>
-      </c>
-      <c r="D12" s="5">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>